<commit_message>
Update Costing Report data to server
</commit_message>
<xml_diff>
--- a/labor_rates.xlsx
+++ b/labor_rates.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\FreeLauncing\Stone River\development\work_pulse_be\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\FreeLauncing\Stone River\development\work_pulse_be\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4823EF5A-582C-40FD-9D03-2E5FE90CB960}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28C9F5B6-974D-40A8-B5A7-1D1E91BC4AF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E075F6AF-0B35-4A2D-B54A-EDC9C634A347}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="19695" windowHeight="15585" xr2:uid="{E075F6AF-0B35-4A2D-B54A-EDC9C634A347}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="15">
   <si>
     <t>TCP</t>
   </si>
@@ -675,7 +675,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D2ED5863-600B-4495-966E-757384B8C73F}">
-  <dimension ref="A1:D50"/>
+  <dimension ref="A1:D51"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="16.85546875" bestFit="1" customWidth="1"/>
@@ -898,10 +898,10 @@
         <v>0</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D16" s="3">
         <v>93.75</v>
@@ -915,7 +915,7 @@
         <v>8</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D17" s="3">
         <v>93.75</v>
@@ -929,7 +929,7 @@
         <v>8</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D18" s="3">
         <v>93.75</v>
@@ -937,16 +937,16 @@
     </row>
     <row r="19" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D19" s="3">
-        <v>67.5</v>
+        <v>93.75</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
@@ -957,10 +957,10 @@
         <v>11</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D20" s="3">
-        <v>81.25</v>
+        <v>67.5</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
@@ -971,10 +971,10 @@
         <v>11</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D21" s="3">
-        <v>105</v>
+        <v>81.25</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
@@ -982,13 +982,13 @@
         <v>9</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D22" s="3">
-        <v>81.25</v>
+        <v>105</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
@@ -999,10 +999,10 @@
         <v>4</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D23" s="3">
-        <v>105</v>
+        <v>81.25</v>
       </c>
     </row>
     <row r="24" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
@@ -1013,7 +1013,7 @@
         <v>4</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D24" s="3">
         <v>105</v>
@@ -1024,13 +1024,13 @@
         <v>9</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D25" s="3">
-        <v>76.88</v>
+        <v>105</v>
       </c>
     </row>
     <row r="26" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
@@ -1041,10 +1041,10 @@
         <v>5</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D26" s="3">
-        <v>94.06</v>
+        <v>76.88</v>
       </c>
     </row>
     <row r="27" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
@@ -1055,10 +1055,10 @@
         <v>5</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D27" s="3">
-        <v>123.75</v>
+        <v>94.06</v>
       </c>
     </row>
     <row r="28" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
@@ -1066,13 +1066,13 @@
         <v>9</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D28" s="3">
-        <v>94.06</v>
+        <v>123.75</v>
       </c>
     </row>
     <row r="29" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
@@ -1083,10 +1083,10 @@
         <v>6</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D29" s="3">
-        <v>123.75</v>
+        <v>94.06</v>
       </c>
     </row>
     <row r="30" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
@@ -1097,7 +1097,7 @@
         <v>6</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D30" s="3">
         <v>123.75</v>
@@ -1108,10 +1108,10 @@
         <v>9</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D31" s="3">
         <v>123.75</v>
@@ -1125,7 +1125,7 @@
         <v>8</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D32" s="3">
         <v>123.75</v>
@@ -1139,7 +1139,7 @@
         <v>8</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D33" s="3">
         <v>123.75</v>
@@ -1147,16 +1147,16 @@
     </row>
     <row r="34" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D34" s="3">
-        <v>88</v>
+        <v>123.75</v>
       </c>
     </row>
     <row r="35" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
@@ -1167,10 +1167,10 @@
         <v>11</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D35" s="3">
-        <v>132</v>
+        <v>88</v>
       </c>
     </row>
     <row r="36" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
@@ -1181,10 +1181,10 @@
         <v>11</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D36" s="3">
-        <v>176</v>
+        <v>132</v>
       </c>
     </row>
     <row r="37" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
@@ -1192,13 +1192,13 @@
         <v>10</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D37" s="3">
-        <v>88</v>
+        <v>176</v>
       </c>
     </row>
     <row r="38" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
@@ -1209,10 +1209,10 @@
         <v>4</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D38" s="3">
-        <v>132</v>
+        <v>88</v>
       </c>
     </row>
     <row r="39" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
@@ -1223,10 +1223,10 @@
         <v>4</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D39" s="3">
-        <v>176</v>
+        <v>132</v>
       </c>
     </row>
     <row r="40" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
@@ -1234,13 +1234,13 @@
         <v>10</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D40" s="3">
-        <v>88</v>
+        <v>176</v>
       </c>
     </row>
     <row r="41" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
@@ -1251,10 +1251,10 @@
         <v>5</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D41" s="3">
-        <v>132</v>
+        <v>88</v>
       </c>
     </row>
     <row r="42" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
@@ -1265,10 +1265,10 @@
         <v>5</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D42" s="3">
-        <v>176</v>
+        <v>132</v>
       </c>
     </row>
     <row r="43" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
@@ -1276,13 +1276,13 @@
         <v>10</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D43" s="3">
-        <v>88</v>
+        <v>176</v>
       </c>
     </row>
     <row r="44" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
@@ -1293,10 +1293,10 @@
         <v>6</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D44" s="3">
-        <v>132</v>
+        <v>88</v>
       </c>
     </row>
     <row r="45" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
@@ -1307,10 +1307,10 @@
         <v>6</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D45" s="3">
-        <v>176</v>
+        <v>132</v>
       </c>
     </row>
     <row r="46" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
@@ -1318,13 +1318,13 @@
         <v>10</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D46" s="3">
-        <v>88</v>
+        <v>176</v>
       </c>
     </row>
     <row r="47" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
@@ -1335,10 +1335,10 @@
         <v>7</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D47" s="3">
-        <v>132</v>
+        <v>88</v>
       </c>
     </row>
     <row r="48" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
@@ -1346,13 +1346,13 @@
         <v>10</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D48" s="3">
-        <v>88</v>
+        <v>132</v>
       </c>
     </row>
     <row r="49" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
@@ -1363,27 +1363,42 @@
         <v>8</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D49" s="3">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A50" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C50" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D50" s="3">
         <v>132</v>
       </c>
     </row>
-    <row r="50" spans="1:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="B50" s="5" t="s">
+    <row r="51" spans="1:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A51" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B51" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C50" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="D50" s="6">
+      <c r="C51" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="D51" s="6">
         <v>176</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>